<commit_message>
Excel analysis, with real data
</commit_message>
<xml_diff>
--- a/tests/sensor-data-2.xlsx
+++ b/tests/sensor-data-2.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tadiwa/Projects/CPRE_288/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9773664F-9D8C-1745-87B4-852D6F036EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F53D2BB-1A32-9C49-9914-F12021C928D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12780" yWindow="4720" windowWidth="28040" windowHeight="17180" xr2:uid="{2AD6BEAB-E07F-A342-AA51-9665AC4D922A}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{2AD6BEAB-E07F-A342-AA51-9665AC4D922A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Real Data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,12 +40,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
     <t>Angle(Degrees)</t>
   </si>
   <si>
     <t>Distance(m)</t>
+  </si>
+  <si>
+    <t>Degrees</t>
+  </si>
+  <si>
+    <t>Distance</t>
   </si>
 </sst>
 </file>
@@ -87,14 +93,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -147,11 +176,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2008,10 +2037,2157 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E92">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="lessThan">
+      <formula>-20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="greaterThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3D5B5AD-62F2-974F-9CD7-E68F6ECF716D}">
+  <dimension ref="A1:K92"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>139</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>63.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>139.1</v>
+      </c>
+      <c r="C3">
+        <f>+B3-B2</f>
+        <v>9.9999999999994316E-2</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>139</v>
+      </c>
+      <c r="J3">
+        <f>+I3-I2</f>
+        <v>75.900000000000006</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>138.6</v>
+      </c>
+      <c r="C4">
+        <f t="shared" ref="C4:C67" si="0">+B4-B3</f>
+        <v>-0.5</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>139.19999999999999</v>
+      </c>
+      <c r="J4">
+        <f t="shared" ref="J4:J67" si="1">+I4-I3</f>
+        <v>0.19999999999998863</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>138.1</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="H5">
+        <v>6</v>
+      </c>
+      <c r="I5">
+        <v>137.6</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="1"/>
+        <v>-1.5999999999999943</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>137.4</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>-0.69999999999998863</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6">
+        <v>138.19999999999999</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="1"/>
+        <v>0.59999999999999432</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>131.1</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>-6.3000000000000114</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>135.80000000000001</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="1"/>
+        <v>-2.3999999999999773</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <v>123.9</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>-7.1999999999999886</v>
+      </c>
+      <c r="H8">
+        <v>12</v>
+      </c>
+      <c r="I8">
+        <v>120.3</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="1"/>
+        <v>-15.500000000000014</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>77.599999999999994</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-46.300000000000011</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>14</v>
+      </c>
+      <c r="I9">
+        <v>81.2</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="1"/>
+        <v>-39.099999999999994</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>72.8</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>-4.7999999999999972</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="H10">
+        <v>16</v>
+      </c>
+      <c r="I10">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="1"/>
+        <v>-10.799999999999997</v>
+      </c>
+      <c r="K10" s="2"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>18</v>
+      </c>
+      <c r="B11">
+        <v>126.9</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>54.100000000000009</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="H11">
+        <v>18</v>
+      </c>
+      <c r="I11">
+        <v>128.19999999999999</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="1"/>
+        <v>57.799999999999983</v>
+      </c>
+      <c r="K11" s="2"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>20</v>
+      </c>
+      <c r="B12">
+        <v>125.1</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>-1.8000000000000114</v>
+      </c>
+      <c r="H12">
+        <v>20</v>
+      </c>
+      <c r="I12">
+        <v>124.3</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="1"/>
+        <v>-3.8999999999999915</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>22</v>
+      </c>
+      <c r="B13">
+        <v>74.3</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>-50.8</v>
+      </c>
+      <c r="D13" s="2">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>22</v>
+      </c>
+      <c r="I13">
+        <v>80.3</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="1"/>
+        <v>-44</v>
+      </c>
+      <c r="K13" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>24</v>
+      </c>
+      <c r="B14">
+        <v>64.3</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>-10</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="H14">
+        <v>24</v>
+      </c>
+      <c r="I14">
+        <v>62.2</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="1"/>
+        <v>-18.099999999999994</v>
+      </c>
+      <c r="K14" s="2"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>26</v>
+      </c>
+      <c r="B15">
+        <v>53.8</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>-10.5</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="H15">
+        <v>26</v>
+      </c>
+      <c r="I15">
+        <v>56.3</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="1"/>
+        <v>-5.9000000000000057</v>
+      </c>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>28</v>
+      </c>
+      <c r="B16">
+        <v>44.6</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>-9.1999999999999957</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="H16">
+        <v>28</v>
+      </c>
+      <c r="I16">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="1"/>
+        <v>-15.5</v>
+      </c>
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>30</v>
+      </c>
+      <c r="B17">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>-3.8000000000000043</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="H17">
+        <v>30</v>
+      </c>
+      <c r="I17">
+        <v>39.1</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="1"/>
+        <v>-1.6999999999999957</v>
+      </c>
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>32</v>
+      </c>
+      <c r="B18">
+        <v>39.1</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>-1.6999999999999957</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="H18">
+        <v>32</v>
+      </c>
+      <c r="I18">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="1"/>
+        <v>-0.39999999999999858</v>
+      </c>
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>34</v>
+      </c>
+      <c r="B19">
+        <v>38.1</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="H19">
+        <v>34</v>
+      </c>
+      <c r="I19">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="1"/>
+        <v>-0.90000000000000568</v>
+      </c>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>36</v>
+      </c>
+      <c r="B20">
+        <v>37.6</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="D20" s="2"/>
+      <c r="H20">
+        <v>36</v>
+      </c>
+      <c r="I20">
+        <v>37.5</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="1"/>
+        <v>-0.29999999999999716</v>
+      </c>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>38</v>
+      </c>
+      <c r="B21">
+        <v>37.9</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>0.29999999999999716</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="H21">
+        <v>38</v>
+      </c>
+      <c r="I21">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="1"/>
+        <v>-0.29999999999999716</v>
+      </c>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>40</v>
+      </c>
+      <c r="B22">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>0.89999999999999858</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="H22">
+        <v>40</v>
+      </c>
+      <c r="I22">
+        <v>38.9</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="1"/>
+        <v>1.6999999999999957</v>
+      </c>
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>42</v>
+      </c>
+      <c r="B23">
+        <v>40.5</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>1.7000000000000028</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="H23">
+        <v>42</v>
+      </c>
+      <c r="I23">
+        <v>39.700000000000003</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="1"/>
+        <v>0.80000000000000426</v>
+      </c>
+      <c r="K23" s="2"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>44</v>
+      </c>
+      <c r="B24">
+        <v>42.2</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="0"/>
+        <v>1.7000000000000028</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="H24">
+        <v>44</v>
+      </c>
+      <c r="I24">
+        <v>43</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="1"/>
+        <v>3.2999999999999972</v>
+      </c>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>46</v>
+      </c>
+      <c r="B25">
+        <v>75.8</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="0"/>
+        <v>33.599999999999994</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="H25">
+        <v>46</v>
+      </c>
+      <c r="I25">
+        <v>75.8</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="1"/>
+        <v>32.799999999999997</v>
+      </c>
+      <c r="K25" s="2"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>48</v>
+      </c>
+      <c r="B26">
+        <v>113.6</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="0"/>
+        <v>37.799999999999997</v>
+      </c>
+      <c r="H26">
+        <v>48</v>
+      </c>
+      <c r="I26">
+        <v>110.9</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="1"/>
+        <v>35.100000000000009</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>50</v>
+      </c>
+      <c r="B27">
+        <v>115.6</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H27">
+        <v>50</v>
+      </c>
+      <c r="I27">
+        <v>118.8</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="1"/>
+        <v>7.8999999999999915</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>52</v>
+      </c>
+      <c r="B28">
+        <v>118.9</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="0"/>
+        <v>3.3000000000000114</v>
+      </c>
+      <c r="H28">
+        <v>52</v>
+      </c>
+      <c r="I28">
+        <v>114.3</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="1"/>
+        <v>-4.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>54</v>
+      </c>
+      <c r="B29">
+        <v>121.2</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="0"/>
+        <v>2.2999999999999972</v>
+      </c>
+      <c r="H29">
+        <v>54</v>
+      </c>
+      <c r="I29">
+        <v>126.9</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="1"/>
+        <v>12.600000000000009</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>56</v>
+      </c>
+      <c r="B30">
+        <v>115.2</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="0"/>
+        <v>-6</v>
+      </c>
+      <c r="H30">
+        <v>56</v>
+      </c>
+      <c r="I30">
+        <v>117.9</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="1"/>
+        <v>-9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>58</v>
+      </c>
+      <c r="B31">
+        <v>109.3</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="0"/>
+        <v>-5.9000000000000057</v>
+      </c>
+      <c r="H31">
+        <v>58</v>
+      </c>
+      <c r="I31">
+        <v>106.4</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="1"/>
+        <v>-11.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>60</v>
+      </c>
+      <c r="B32">
+        <v>101.6</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="0"/>
+        <v>-7.7000000000000028</v>
+      </c>
+      <c r="H32">
+        <v>60</v>
+      </c>
+      <c r="I32">
+        <v>136.19999999999999</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="1"/>
+        <v>29.799999999999983</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>62</v>
+      </c>
+      <c r="B33">
+        <v>89.7</v>
+      </c>
+      <c r="C33">
+        <f t="shared" si="0"/>
+        <v>-11.899999999999991</v>
+      </c>
+      <c r="H33">
+        <v>62</v>
+      </c>
+      <c r="I33">
+        <v>89.1</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="1"/>
+        <v>-47.099999999999994</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>64</v>
+      </c>
+      <c r="B34">
+        <v>88.7</v>
+      </c>
+      <c r="C34">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="H34">
+        <v>64</v>
+      </c>
+      <c r="I34">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="1"/>
+        <v>-10.699999999999989</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>66</v>
+      </c>
+      <c r="B35">
+        <v>96.3</v>
+      </c>
+      <c r="C35">
+        <f t="shared" si="0"/>
+        <v>7.5999999999999943</v>
+      </c>
+      <c r="H35">
+        <v>66</v>
+      </c>
+      <c r="I35">
+        <v>98.1</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="1"/>
+        <v>19.699999999999989</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>68</v>
+      </c>
+      <c r="B36">
+        <v>105.7</v>
+      </c>
+      <c r="C36">
+        <f t="shared" si="0"/>
+        <v>9.4000000000000057</v>
+      </c>
+      <c r="H36">
+        <v>68</v>
+      </c>
+      <c r="I36">
+        <v>102</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="1"/>
+        <v>3.9000000000000057</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>70</v>
+      </c>
+      <c r="B37">
+        <v>114</v>
+      </c>
+      <c r="C37">
+        <f t="shared" si="0"/>
+        <v>8.2999999999999972</v>
+      </c>
+      <c r="H37">
+        <v>70</v>
+      </c>
+      <c r="I37">
+        <v>118.8</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="1"/>
+        <v>16.799999999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>72</v>
+      </c>
+      <c r="B38">
+        <v>116.3</v>
+      </c>
+      <c r="C38">
+        <f t="shared" si="0"/>
+        <v>2.2999999999999972</v>
+      </c>
+      <c r="H38">
+        <v>72</v>
+      </c>
+      <c r="I38">
+        <v>117.4</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="1"/>
+        <v>-1.3999999999999915</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>74</v>
+      </c>
+      <c r="B39">
+        <v>28.3</v>
+      </c>
+      <c r="C39">
+        <f t="shared" si="0"/>
+        <v>-88</v>
+      </c>
+      <c r="D39" s="2">
+        <v>3</v>
+      </c>
+      <c r="H39">
+        <v>74</v>
+      </c>
+      <c r="I39">
+        <v>26.4</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="1"/>
+        <v>-91</v>
+      </c>
+      <c r="K39" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>76</v>
+      </c>
+      <c r="B40">
+        <v>31.8</v>
+      </c>
+      <c r="C40">
+        <f t="shared" si="0"/>
+        <v>3.5</v>
+      </c>
+      <c r="D40" s="2"/>
+      <c r="H40">
+        <v>76</v>
+      </c>
+      <c r="I40">
+        <v>32.1</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="1"/>
+        <v>5.7000000000000028</v>
+      </c>
+      <c r="K40" s="2"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>78</v>
+      </c>
+      <c r="B41">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="0"/>
+        <v>1.4999999999999964</v>
+      </c>
+      <c r="D41" s="2"/>
+      <c r="H41">
+        <v>78</v>
+      </c>
+      <c r="I41">
+        <v>34.9</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="1"/>
+        <v>2.7999999999999972</v>
+      </c>
+      <c r="K41" s="2"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>80</v>
+      </c>
+      <c r="B42">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="0"/>
+        <v>-9.9999999999994316E-2</v>
+      </c>
+      <c r="D42" s="2"/>
+      <c r="H42">
+        <v>80</v>
+      </c>
+      <c r="I42">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="1"/>
+        <v>-1.6000000000000014</v>
+      </c>
+      <c r="K42" s="2"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>82</v>
+      </c>
+      <c r="B43">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="C43">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="D43" s="2"/>
+      <c r="H43">
+        <v>82</v>
+      </c>
+      <c r="I43">
+        <v>33</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="1"/>
+        <v>-0.29999999999999716</v>
+      </c>
+      <c r="K43" s="2"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>84</v>
+      </c>
+      <c r="B44">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="C44">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="D44" s="2"/>
+      <c r="H44">
+        <v>84</v>
+      </c>
+      <c r="I44">
+        <v>34.700000000000003</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="1"/>
+        <v>1.7000000000000028</v>
+      </c>
+      <c r="K44" s="2"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>86</v>
+      </c>
+      <c r="B45">
+        <v>32.4</v>
+      </c>
+      <c r="C45">
+        <f t="shared" si="0"/>
+        <v>-0.80000000000000426</v>
+      </c>
+      <c r="D45" s="2"/>
+      <c r="H45">
+        <v>86</v>
+      </c>
+      <c r="I45">
+        <v>31.2</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="1"/>
+        <v>-3.5000000000000036</v>
+      </c>
+      <c r="K45" s="2"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>88</v>
+      </c>
+      <c r="B46">
+        <v>32.6</v>
+      </c>
+      <c r="C46">
+        <f t="shared" si="0"/>
+        <v>0.20000000000000284</v>
+      </c>
+      <c r="D46" s="2"/>
+      <c r="H46">
+        <v>88</v>
+      </c>
+      <c r="I46">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="1"/>
+        <v>1.5999999999999979</v>
+      </c>
+      <c r="K46" s="2"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>90</v>
+      </c>
+      <c r="B47">
+        <v>135.30000000000001</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="0"/>
+        <v>102.70000000000002</v>
+      </c>
+      <c r="D47" s="2"/>
+      <c r="H47">
+        <v>90</v>
+      </c>
+      <c r="I47">
+        <v>133.80000000000001</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="1"/>
+        <v>101.00000000000001</v>
+      </c>
+      <c r="K47" s="2"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>92</v>
+      </c>
+      <c r="B48">
+        <v>137.4</v>
+      </c>
+      <c r="C48">
+        <f t="shared" si="0"/>
+        <v>2.0999999999999943</v>
+      </c>
+      <c r="H48">
+        <v>92</v>
+      </c>
+      <c r="I48">
+        <v>138.19999999999999</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="1"/>
+        <v>4.3999999999999773</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>94</v>
+      </c>
+      <c r="B49">
+        <v>138.1</v>
+      </c>
+      <c r="C49">
+        <f t="shared" si="0"/>
+        <v>0.69999999999998863</v>
+      </c>
+      <c r="H49">
+        <v>94</v>
+      </c>
+      <c r="I49">
+        <v>138.6</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="1"/>
+        <v>0.40000000000000568</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>96</v>
+      </c>
+      <c r="B50">
+        <v>137.69999999999999</v>
+      </c>
+      <c r="C50">
+        <f t="shared" si="0"/>
+        <v>-0.40000000000000568</v>
+      </c>
+      <c r="H50">
+        <v>96</v>
+      </c>
+      <c r="I50">
+        <v>138.19999999999999</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="1"/>
+        <v>-0.40000000000000568</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>98</v>
+      </c>
+      <c r="B51">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="C51">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="H51">
+        <v>98</v>
+      </c>
+      <c r="I51">
+        <v>136.80000000000001</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="1"/>
+        <v>-1.3999999999999773</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>100</v>
+      </c>
+      <c r="B52">
+        <v>137.5</v>
+      </c>
+      <c r="C52">
+        <f t="shared" si="0"/>
+        <v>0.30000000000001137</v>
+      </c>
+      <c r="H52">
+        <v>100</v>
+      </c>
+      <c r="I52">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="1"/>
+        <v>0.39999999999997726</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>102</v>
+      </c>
+      <c r="B53">
+        <v>138.19999999999999</v>
+      </c>
+      <c r="C53">
+        <f t="shared" si="0"/>
+        <v>0.69999999999998863</v>
+      </c>
+      <c r="H53">
+        <v>102</v>
+      </c>
+      <c r="I53">
+        <v>138.19999999999999</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>104</v>
+      </c>
+      <c r="B54">
+        <v>138</v>
+      </c>
+      <c r="C54">
+        <f t="shared" si="0"/>
+        <v>-0.19999999999998863</v>
+      </c>
+      <c r="H54">
+        <v>104</v>
+      </c>
+      <c r="I54">
+        <v>138.80000000000001</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="1"/>
+        <v>0.60000000000002274</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>106</v>
+      </c>
+      <c r="B55">
+        <v>137.9</v>
+      </c>
+      <c r="C55">
+        <f t="shared" si="0"/>
+        <v>-9.9999999999994316E-2</v>
+      </c>
+      <c r="H55">
+        <v>106</v>
+      </c>
+      <c r="I55">
+        <v>137</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="1"/>
+        <v>-1.8000000000000114</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>108</v>
+      </c>
+      <c r="B56">
+        <v>137.6</v>
+      </c>
+      <c r="C56">
+        <f t="shared" si="0"/>
+        <v>-0.30000000000001137</v>
+      </c>
+      <c r="H56">
+        <v>108</v>
+      </c>
+      <c r="I56">
+        <v>138.80000000000001</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="1"/>
+        <v>1.8000000000000114</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>110</v>
+      </c>
+      <c r="B57">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="C57">
+        <f t="shared" si="0"/>
+        <v>-0.40000000000000568</v>
+      </c>
+      <c r="H57">
+        <v>110</v>
+      </c>
+      <c r="I57">
+        <v>136.19999999999999</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="1"/>
+        <v>-2.6000000000000227</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>112</v>
+      </c>
+      <c r="B58">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="C58">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <v>112</v>
+      </c>
+      <c r="I58">
+        <v>137.80000000000001</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="1"/>
+        <v>1.6000000000000227</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>114</v>
+      </c>
+      <c r="B59">
+        <v>137</v>
+      </c>
+      <c r="C59">
+        <f t="shared" si="0"/>
+        <v>-0.19999999999998863</v>
+      </c>
+      <c r="H59">
+        <v>114</v>
+      </c>
+      <c r="I59">
+        <v>136.6</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="1"/>
+        <v>-1.2000000000000171</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>116</v>
+      </c>
+      <c r="B60">
+        <v>136.9</v>
+      </c>
+      <c r="C60">
+        <f t="shared" si="0"/>
+        <v>-9.9999999999994316E-2</v>
+      </c>
+      <c r="H60">
+        <v>116</v>
+      </c>
+      <c r="I60">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="1"/>
+        <v>0.59999999999999432</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>118</v>
+      </c>
+      <c r="B61">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="C61">
+        <f t="shared" si="0"/>
+        <v>0.29999999999998295</v>
+      </c>
+      <c r="H61">
+        <v>118</v>
+      </c>
+      <c r="I61">
+        <v>136.4</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="1"/>
+        <v>-0.79999999999998295</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>120</v>
+      </c>
+      <c r="B62">
+        <v>138</v>
+      </c>
+      <c r="C62">
+        <f t="shared" si="0"/>
+        <v>0.80000000000001137</v>
+      </c>
+      <c r="H62">
+        <v>120</v>
+      </c>
+      <c r="I62">
+        <v>138.4</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>122</v>
+      </c>
+      <c r="B63">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="C63">
+        <f t="shared" si="0"/>
+        <v>-105.2</v>
+      </c>
+      <c r="D63" s="2">
+        <v>4</v>
+      </c>
+      <c r="H63">
+        <v>122</v>
+      </c>
+      <c r="I63">
+        <v>31.9</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="1"/>
+        <v>-106.5</v>
+      </c>
+      <c r="K63" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>124</v>
+      </c>
+      <c r="B64">
+        <v>35.299999999999997</v>
+      </c>
+      <c r="C64">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="D64" s="2"/>
+      <c r="H64">
+        <v>124</v>
+      </c>
+      <c r="I64">
+        <v>34.5</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="1"/>
+        <v>2.6000000000000014</v>
+      </c>
+      <c r="K64" s="2"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>126</v>
+      </c>
+      <c r="B65">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="C65">
+        <f t="shared" si="0"/>
+        <v>1.9000000000000057</v>
+      </c>
+      <c r="D65" s="2"/>
+      <c r="H65">
+        <v>126</v>
+      </c>
+      <c r="I65">
+        <v>38.6</v>
+      </c>
+      <c r="J65">
+        <f t="shared" si="1"/>
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="K65" s="2"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>128</v>
+      </c>
+      <c r="B66">
+        <v>37.1</v>
+      </c>
+      <c r="C66">
+        <f t="shared" si="0"/>
+        <v>-0.10000000000000142</v>
+      </c>
+      <c r="D66" s="2"/>
+      <c r="H66">
+        <v>128</v>
+      </c>
+      <c r="I66">
+        <v>37.700000000000003</v>
+      </c>
+      <c r="J66">
+        <f t="shared" si="1"/>
+        <v>-0.89999999999999858</v>
+      </c>
+      <c r="K66" s="2"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>130</v>
+      </c>
+      <c r="B67">
+        <v>36.1</v>
+      </c>
+      <c r="C67">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="D67" s="2"/>
+      <c r="H67">
+        <v>130</v>
+      </c>
+      <c r="I67">
+        <v>36.5</v>
+      </c>
+      <c r="J67">
+        <f t="shared" si="1"/>
+        <v>-1.2000000000000028</v>
+      </c>
+      <c r="K67" s="2"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>132</v>
+      </c>
+      <c r="B68">
+        <v>35</v>
+      </c>
+      <c r="C68">
+        <f t="shared" ref="C68:C92" si="2">+B68-B67</f>
+        <v>-1.1000000000000014</v>
+      </c>
+      <c r="D68" s="2"/>
+      <c r="H68">
+        <v>132</v>
+      </c>
+      <c r="I68">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="J68">
+        <f t="shared" ref="J68:J92" si="3">+I68-I67</f>
+        <v>-1.7000000000000028</v>
+      </c>
+      <c r="K68" s="2"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>134</v>
+      </c>
+      <c r="B69">
+        <v>34.6</v>
+      </c>
+      <c r="C69">
+        <f t="shared" si="2"/>
+        <v>-0.39999999999999858</v>
+      </c>
+      <c r="D69" s="2"/>
+      <c r="H69">
+        <v>134</v>
+      </c>
+      <c r="I69">
+        <v>34</v>
+      </c>
+      <c r="J69">
+        <f t="shared" si="3"/>
+        <v>-0.79999999999999716</v>
+      </c>
+      <c r="K69" s="2"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>136</v>
+      </c>
+      <c r="B70">
+        <v>34.6</v>
+      </c>
+      <c r="C70">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D70" s="2"/>
+      <c r="H70">
+        <v>136</v>
+      </c>
+      <c r="I70">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="J70">
+        <f t="shared" si="3"/>
+        <v>0.79999999999999716</v>
+      </c>
+      <c r="K70" s="2"/>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>138</v>
+      </c>
+      <c r="B71">
+        <v>35</v>
+      </c>
+      <c r="C71">
+        <f t="shared" si="2"/>
+        <v>0.39999999999999858</v>
+      </c>
+      <c r="D71" s="2"/>
+      <c r="H71">
+        <v>138</v>
+      </c>
+      <c r="I71">
+        <v>34.6</v>
+      </c>
+      <c r="J71">
+        <f t="shared" si="3"/>
+        <v>-0.19999999999999574</v>
+      </c>
+      <c r="K71" s="2"/>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>140</v>
+      </c>
+      <c r="B72">
+        <v>36.200000000000003</v>
+      </c>
+      <c r="C72">
+        <f t="shared" si="2"/>
+        <v>1.2000000000000028</v>
+      </c>
+      <c r="D72" s="2"/>
+      <c r="H72">
+        <v>140</v>
+      </c>
+      <c r="I72">
+        <v>35.9</v>
+      </c>
+      <c r="J72">
+        <f t="shared" si="3"/>
+        <v>1.2999999999999972</v>
+      </c>
+      <c r="K72" s="2"/>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>142</v>
+      </c>
+      <c r="B73">
+        <v>37.4</v>
+      </c>
+      <c r="C73">
+        <f t="shared" si="2"/>
+        <v>1.1999999999999957</v>
+      </c>
+      <c r="D73" s="2"/>
+      <c r="H73">
+        <v>142</v>
+      </c>
+      <c r="I73">
+        <v>37.6</v>
+      </c>
+      <c r="J73">
+        <f t="shared" si="3"/>
+        <v>1.7000000000000028</v>
+      </c>
+      <c r="K73" s="2"/>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>144</v>
+      </c>
+      <c r="B74">
+        <v>42.9</v>
+      </c>
+      <c r="C74">
+        <f t="shared" si="2"/>
+        <v>5.5</v>
+      </c>
+      <c r="D74" s="2"/>
+      <c r="H74">
+        <v>144</v>
+      </c>
+      <c r="I74">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="J74">
+        <f t="shared" si="3"/>
+        <v>0.69999999999999574</v>
+      </c>
+      <c r="K74" s="2"/>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>146</v>
+      </c>
+      <c r="B75">
+        <v>49.8</v>
+      </c>
+      <c r="C75">
+        <f t="shared" si="2"/>
+        <v>6.8999999999999986</v>
+      </c>
+      <c r="D75" s="2"/>
+      <c r="H75">
+        <v>146</v>
+      </c>
+      <c r="I75">
+        <v>53.2</v>
+      </c>
+      <c r="J75">
+        <f t="shared" si="3"/>
+        <v>14.900000000000006</v>
+      </c>
+      <c r="K75" s="2"/>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>148</v>
+      </c>
+      <c r="B76">
+        <v>98.1</v>
+      </c>
+      <c r="C76">
+        <f t="shared" si="2"/>
+        <v>48.3</v>
+      </c>
+      <c r="D76" s="2"/>
+      <c r="H76">
+        <v>148</v>
+      </c>
+      <c r="I76">
+        <v>98.1</v>
+      </c>
+      <c r="J76">
+        <f t="shared" si="3"/>
+        <v>44.899999999999991</v>
+      </c>
+      <c r="K76" s="2"/>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>150</v>
+      </c>
+      <c r="B77">
+        <v>124.3</v>
+      </c>
+      <c r="C77">
+        <f t="shared" si="2"/>
+        <v>26.200000000000003</v>
+      </c>
+      <c r="H77">
+        <v>150</v>
+      </c>
+      <c r="I77">
+        <v>127.1</v>
+      </c>
+      <c r="J77">
+        <f t="shared" si="3"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>152</v>
+      </c>
+      <c r="B78">
+        <v>120.7</v>
+      </c>
+      <c r="C78">
+        <f t="shared" si="2"/>
+        <v>-3.5999999999999943</v>
+      </c>
+      <c r="H78">
+        <v>152</v>
+      </c>
+      <c r="I78">
+        <v>118.8</v>
+      </c>
+      <c r="J78">
+        <f t="shared" si="3"/>
+        <v>-8.2999999999999972</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A79">
+        <v>154</v>
+      </c>
+      <c r="B79">
+        <v>132.30000000000001</v>
+      </c>
+      <c r="C79">
+        <f t="shared" si="2"/>
+        <v>11.600000000000009</v>
+      </c>
+      <c r="H79">
+        <v>154</v>
+      </c>
+      <c r="I79">
+        <v>139</v>
+      </c>
+      <c r="J79">
+        <f t="shared" si="3"/>
+        <v>20.200000000000003</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A80">
+        <v>156</v>
+      </c>
+      <c r="B80">
+        <v>135.6</v>
+      </c>
+      <c r="C80">
+        <f t="shared" si="2"/>
+        <v>3.2999999999999829</v>
+      </c>
+      <c r="H80">
+        <v>156</v>
+      </c>
+      <c r="I80">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="J80">
+        <f t="shared" si="3"/>
+        <v>-1.8000000000000114</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>158</v>
+      </c>
+      <c r="B81">
+        <v>134.19999999999999</v>
+      </c>
+      <c r="C81">
+        <f t="shared" si="2"/>
+        <v>-1.4000000000000057</v>
+      </c>
+      <c r="H81">
+        <v>158</v>
+      </c>
+      <c r="I81">
+        <v>137.19999999999999</v>
+      </c>
+      <c r="J81">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>160</v>
+      </c>
+      <c r="B82">
+        <v>131.9</v>
+      </c>
+      <c r="C82">
+        <f t="shared" si="2"/>
+        <v>-2.2999999999999829</v>
+      </c>
+      <c r="H82">
+        <v>160</v>
+      </c>
+      <c r="I82">
+        <v>129.9</v>
+      </c>
+      <c r="J82">
+        <f t="shared" si="3"/>
+        <v>-7.2999999999999829</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>162</v>
+      </c>
+      <c r="B83">
+        <v>131.69999999999999</v>
+      </c>
+      <c r="C83">
+        <f t="shared" si="2"/>
+        <v>-0.20000000000001705</v>
+      </c>
+      <c r="H83">
+        <v>162</v>
+      </c>
+      <c r="I83">
+        <v>131.6</v>
+      </c>
+      <c r="J83">
+        <f t="shared" si="3"/>
+        <v>1.6999999999999886</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>164</v>
+      </c>
+      <c r="B84">
+        <v>111.1</v>
+      </c>
+      <c r="C84">
+        <f t="shared" si="2"/>
+        <v>-20.599999999999994</v>
+      </c>
+      <c r="H84">
+        <v>164</v>
+      </c>
+      <c r="I84">
+        <v>111.1</v>
+      </c>
+      <c r="J84">
+        <f t="shared" si="3"/>
+        <v>-20.5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>166</v>
+      </c>
+      <c r="B85">
+        <v>35.4</v>
+      </c>
+      <c r="C85">
+        <f t="shared" si="2"/>
+        <v>-75.699999999999989</v>
+      </c>
+      <c r="D85" s="1"/>
+      <c r="H85">
+        <v>166</v>
+      </c>
+      <c r="I85">
+        <v>33.9</v>
+      </c>
+      <c r="J85">
+        <f t="shared" si="3"/>
+        <v>-77.199999999999989</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>168</v>
+      </c>
+      <c r="B86">
+        <v>38.4</v>
+      </c>
+      <c r="C86">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="D86" s="1"/>
+      <c r="H86">
+        <v>168</v>
+      </c>
+      <c r="I86">
+        <v>38.200000000000003</v>
+      </c>
+      <c r="J86">
+        <f t="shared" si="3"/>
+        <v>4.3000000000000043</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>170</v>
+      </c>
+      <c r="B87">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="C87">
+        <f t="shared" si="2"/>
+        <v>2.3000000000000043</v>
+      </c>
+      <c r="D87" s="1"/>
+      <c r="H87">
+        <v>170</v>
+      </c>
+      <c r="I87">
+        <v>41.7</v>
+      </c>
+      <c r="J87">
+        <f t="shared" si="3"/>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>172</v>
+      </c>
+      <c r="B88">
+        <v>41.2</v>
+      </c>
+      <c r="C88">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="D88" s="1"/>
+      <c r="H88">
+        <v>172</v>
+      </c>
+      <c r="I88">
+        <v>42.1</v>
+      </c>
+      <c r="J88">
+        <f t="shared" si="3"/>
+        <v>0.39999999999999858</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>174</v>
+      </c>
+      <c r="B89">
+        <v>40.9</v>
+      </c>
+      <c r="C89">
+        <f t="shared" si="2"/>
+        <v>-0.30000000000000426</v>
+      </c>
+      <c r="D89" s="1"/>
+      <c r="H89">
+        <v>174</v>
+      </c>
+      <c r="I89">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="J89">
+        <f t="shared" si="3"/>
+        <v>-1.3999999999999986</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>176</v>
+      </c>
+      <c r="B90">
+        <v>41</v>
+      </c>
+      <c r="C90">
+        <f t="shared" si="2"/>
+        <v>0.10000000000000142</v>
+      </c>
+      <c r="D90" s="1"/>
+      <c r="H90">
+        <v>176</v>
+      </c>
+      <c r="I90">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="J90">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>178</v>
+      </c>
+      <c r="B91">
+        <v>41.6</v>
+      </c>
+      <c r="C91">
+        <f t="shared" si="2"/>
+        <v>0.60000000000000142</v>
+      </c>
+      <c r="D91" s="1"/>
+      <c r="H91">
+        <v>178</v>
+      </c>
+      <c r="I91">
+        <v>41.5</v>
+      </c>
+      <c r="J91">
+        <f t="shared" si="3"/>
+        <v>0.79999999999999716</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>180</v>
+      </c>
+      <c r="B92">
+        <v>42</v>
+      </c>
+      <c r="C92">
+        <f t="shared" si="2"/>
+        <v>0.39999999999999858</v>
+      </c>
+      <c r="D92" s="1"/>
+      <c r="H92">
+        <v>180</v>
+      </c>
+      <c r="I92">
+        <v>42.2</v>
+      </c>
+      <c r="J92">
+        <f t="shared" si="3"/>
+        <v>0.70000000000000284</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="K9:K11"/>
+    <mergeCell ref="K13:K25"/>
+    <mergeCell ref="K39:K47"/>
+    <mergeCell ref="K63:K76"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="D13:D25"/>
+    <mergeCell ref="D39:D47"/>
+    <mergeCell ref="D63:D76"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C3:C92">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThan">
+      <formula>-20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J92">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>-20</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>